<commit_message>
Update Day 1 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7230D95-A338-496A-BD03-AAC1FE223356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC6C0A4-6854-493F-AE0B-275268166A0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t>MCA - D1P2633</t>
+  </si>
+  <si>
+    <t>Practicals and focused study</t>
   </si>
 </sst>
 </file>
@@ -723,25 +726,47 @@
       <ns0:c r="A6" s="3">
         <ns0:v>46247</ns0:v>
       </ns0:c>
-      <ns0:c r="B6" s="4"/>
-      <ns0:c r="C6" s="4"/>
-      <ns0:c r="D6" s="4"/>
-      <ns0:c r="E6" s="4"/>
-      <ns0:c r="F6" s="4"/>
-      <ns0:c r="G6" s="4"/>
-      <ns0:c r="H6" s="4"/>
-      <ns0:c r="I6" s="5" t="str">
+      <ns0:c r="B6" s="4">
+        <ns0:v>560</ns0:v>
+      </ns0:c>
+      <ns0:c r="C6" s="4">
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="D6" s="4">
+        <ns0:v>70</ns0:v>
+      </ns0:c>
+      <ns0:c r="E6" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="F6" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="G6" s="4">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="H6" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I6" s="5">
         <ns0:f>IF(COUNT(B6:F6,H6)&lt;6,"",SUM(B6:F6,H6))</ns0:f>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J6" s="5" t="str">
+        <ns0:v>1430</ns0:v>
+      </ns0:c>
+      <ns0:c r="J6" s="5">
         <ns0:f>IF(I6="","",1440-I6)</ns0:f>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K6" s="4"/>
-      <ns0:c r="L6" s="4"/>
-      <ns0:c r="M6" s="4"/>
-      <ns0:c r="N6" s="6"/>
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="K6" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L6" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M6" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N6" s="4" t="s">
+        <ns0:v>36</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="7" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A7" s="3">

</xml_diff>

<commit_message>
Update Day 2 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC6C0A4-6854-493F-AE0B-275268166A0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBEAD465-6672-47B9-AEA4-796D0288BBD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -168,6 +168,9 @@
   </si>
   <si>
     <t>Practicals and focused study</t>
+  </si>
+  <si>
+    <t>Balanced</t>
   </si>
 </sst>
 </file>
@@ -772,25 +775,47 @@
       <ns0:c r="A7" s="3">
         <ns0:v>46248</ns0:v>
       </ns0:c>
-      <ns0:c r="B7" s="4"/>
-      <ns0:c r="C7" s="13"/>
-      <ns0:c r="D7" s="13"/>
-      <ns0:c r="E7" s="13"/>
-      <ns0:c r="F7" s="13"/>
-      <ns0:c r="G7" s="13"/>
-      <ns0:c r="H7" s="13"/>
-      <ns0:c r="I7" s="5" t="str">
+      <ns0:c r="B7" s="4">
+        <ns0:v>530</ns0:v>
+      </ns0:c>
+      <ns0:c r="C7" s="4">
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="D7" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="E7" s="4">
+        <ns0:v>260</ns0:v>
+      </ns0:c>
+      <ns0:c r="F7" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G7" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H7" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I7" s="5">
         <ns0:f t="shared" ref="I7:I12" si="0">IF(COUNT(B7:F7,H7)&lt;6,"",SUM(B7:F7,H7))</ns0:f>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J7" s="5" t="str">
+        <ns0:v>1400</ns0:v>
+      </ns0:c>
+      <ns0:c r="J7" s="5">
         <ns0:f t="shared" ref="J7:J12" si="1">IF(I7="","",1440-I7)</ns0:f>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K7" s="4"/>
-      <ns0:c r="L7" s="4"/>
-      <ns0:c r="M7" s="4"/>
-      <ns0:c r="N7" s="6"/>
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="K7" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L7" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M7" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N7" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="8" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A8" s="3">

</xml_diff>

<commit_message>
Update Day 3 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBEAD465-6672-47B9-AEA4-796D0288BBD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B26C58-41CA-422C-A72F-27C4CD829949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -171,6 +171,9 @@
   </si>
   <si>
     <t>Balanced</t>
+  </si>
+  <si>
+    <t>Project work and revision</t>
   </si>
 </sst>
 </file>
@@ -821,25 +824,47 @@
       <ns0:c r="A8" s="3">
         <ns0:v>46249</ns0:v>
       </ns0:c>
-      <ns0:c r="B8" s="4"/>
-      <ns0:c r="C8" s="13"/>
-      <ns0:c r="D8" s="13"/>
-      <ns0:c r="E8" s="13"/>
-      <ns0:c r="F8" s="13"/>
-      <ns0:c r="G8" s="13"/>
-      <ns0:c r="H8" s="13"/>
-      <ns0:c r="I8" s="5" t="str">
+      <ns0:c r="B8" s="4">
+        <ns0:v>520</ns0:v>
+      </ns0:c>
+      <ns0:c r="C8" s="4">
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="D8" s="4">
+        <ns0:v>170</ns0:v>
+      </ns0:c>
+      <ns0:c r="E8" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="F8" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="G8" s="4">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="H8" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I8" s="5">
         <ns0:f t="shared" si="0"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J8" s="5" t="str">
+        <ns0:v>1350</ns0:v>
+      </ns0:c>
+      <ns0:c r="J8" s="5">
         <ns0:f t="shared" si="1"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K8" s="4"/>
-      <ns0:c r="L8" s="4"/>
-      <ns0:c r="M8" s="4"/>
-      <ns0:c r="N8" s="6"/>
+        <ns0:v>90</ns0:v>
+      </ns0:c>
+      <ns0:c r="K8" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L8" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M8" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N8" s="4" t="s">
+        <ns0:v>38</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="9" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A9" s="3">

</xml_diff>

<commit_message>
Update Day 4 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B26C58-41CA-422C-A72F-27C4CD829949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CD2EC3E-C179-493E-ACFD-9D75F976A183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -174,6 +174,9 @@
   </si>
   <si>
     <t>Project work and revision</t>
+  </si>
+  <si>
+    <t>Rest, notes and planning</t>
   </si>
 </sst>
 </file>
@@ -870,25 +873,47 @@
       <ns0:c r="A9" s="3">
         <ns0:v>46250</ns0:v>
       </ns0:c>
-      <ns0:c r="B9" s="4"/>
-      <ns0:c r="C9" s="13"/>
-      <ns0:c r="D9" s="13"/>
-      <ns0:c r="E9" s="13"/>
-      <ns0:c r="F9" s="13"/>
-      <ns0:c r="G9" s="13"/>
-      <ns0:c r="H9" s="13"/>
-      <ns0:c r="I9" s="5" t="str">
+      <ns0:c r="B9" s="4">
+        <ns0:v>560</ns0:v>
+      </ns0:c>
+      <ns0:c r="C9" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D9" s="4">
+        <ns0:v>130</ns0:v>
+      </ns0:c>
+      <ns0:c r="E9" s="4">
+        <ns0:v>410</ns0:v>
+      </ns0:c>
+      <ns0:c r="F9" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="G9" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="H9" s="4">
+        <ns0:v>280</ns0:v>
+      </ns0:c>
+      <ns0:c r="I9" s="5">
         <ns0:f t="shared" si="0"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J9" s="5" t="str">
+        <ns0:v>1410</ns0:v>
+      </ns0:c>
+      <ns0:c r="J9" s="5">
         <ns0:f t="shared" si="1"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K9" s="4"/>
-      <ns0:c r="L9" s="4"/>
-      <ns0:c r="M9" s="4"/>
-      <ns0:c r="N9" s="6"/>
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="K9" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L9" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M9" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N9" s="4" t="s">
+        <ns0:v>39</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="10" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A10" s="3">

</xml_diff>

<commit_message>
Update Day 5 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CD2EC3E-C179-493E-ACFD-9D75F976A183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52FAB1A1-2E1B-410C-902A-C9E9BC7016D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -919,25 +919,47 @@
       <ns0:c r="A10" s="3">
         <ns0:v>46251</ns0:v>
       </ns0:c>
-      <ns0:c r="B10" s="4"/>
-      <ns0:c r="C10" s="13"/>
-      <ns0:c r="D10" s="13"/>
-      <ns0:c r="E10" s="13"/>
-      <ns0:c r="F10" s="13"/>
-      <ns0:c r="G10" s="13"/>
-      <ns0:c r="H10" s="13"/>
-      <ns0:c r="I10" s="5" t="str">
+      <ns0:c r="B10" s="4">
+        <ns0:v>560</ns0:v>
+      </ns0:c>
+      <ns0:c r="C10" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D10" s="4">
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="E10" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="F10" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G10" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H10" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I10" s="5">
         <ns0:f t="shared" si="0"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J10" s="5" t="str">
+        <ns0:v>1360</ns0:v>
+      </ns0:c>
+      <ns0:c r="J10" s="5">
         <ns0:f t="shared" si="1"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K10" s="4"/>
-      <ns0:c r="L10" s="4"/>
-      <ns0:c r="M10" s="4"/>
-      <ns0:c r="N10" s="6"/>
+        <ns0:v>80</ns0:v>
+      </ns0:c>
+      <ns0:c r="K10" s="4" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="L10" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M10" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N10" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="11" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A11" s="3">

</xml_diff>

<commit_message>
Update Day 6 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52FAB1A1-2E1B-410C-902A-C9E9BC7016D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8FF0E4-BA70-4783-A687-88F5F5440788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="41">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -177,6 +177,9 @@
   </si>
   <si>
     <t>Rest, notes and planning</t>
+  </si>
+  <si>
+    <t>Balanced day with practicals</t>
   </si>
 </sst>
 </file>
@@ -965,25 +968,47 @@
       <ns0:c r="A11" s="3">
         <ns0:v>46252</ns0:v>
       </ns0:c>
-      <ns0:c r="B11" s="4"/>
-      <ns0:c r="C11" s="13"/>
-      <ns0:c r="D11" s="13"/>
-      <ns0:c r="E11" s="13"/>
-      <ns0:c r="F11" s="13"/>
-      <ns0:c r="G11" s="13"/>
-      <ns0:c r="H11" s="13"/>
-      <ns0:c r="I11" s="5" t="str">
+      <ns0:c r="B11" s="4">
+        <ns0:v>520</ns0:v>
+      </ns0:c>
+      <ns0:c r="C11" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D11" s="4">
+        <ns0:v>110</ns0:v>
+      </ns0:c>
+      <ns0:c r="E11" s="4">
+        <ns0:v>260</ns0:v>
+      </ns0:c>
+      <ns0:c r="F11" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G11" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H11" s="4">
+        <ns0:v>260</ns0:v>
+      </ns0:c>
+      <ns0:c r="I11" s="5">
         <ns0:f t="shared" si="0"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J11" s="5" t="str">
+        <ns0:v>1440</ns0:v>
+      </ns0:c>
+      <ns0:c r="J11" s="5">
         <ns0:f t="shared" si="1"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K11" s="4"/>
-      <ns0:c r="L11" s="4"/>
-      <ns0:c r="M11" s="4"/>
-      <ns0:c r="N11" s="6"/>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K11" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L11" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M11" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N11" s="4" t="s">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="12" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A12" s="3">

</xml_diff>

<commit_message>
Update Day 7 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8FF0E4-BA70-4783-A687-88F5F5440788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0302D5C8-EA0F-436E-A85F-12BE17B0D05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -180,6 +180,9 @@
   </si>
   <si>
     <t>Balanced day with practicals</t>
+  </si>
+  <si>
+    <t>Steady progress</t>
   </si>
 </sst>
 </file>
@@ -1014,25 +1017,47 @@
       <ns0:c r="A12" s="3">
         <ns0:v>46253</ns0:v>
       </ns0:c>
-      <ns0:c r="B12" s="4"/>
-      <ns0:c r="C12" s="13"/>
-      <ns0:c r="D12" s="13"/>
-      <ns0:c r="E12" s="13"/>
-      <ns0:c r="F12" s="13"/>
-      <ns0:c r="G12" s="13"/>
-      <ns0:c r="H12" s="13"/>
-      <ns0:c r="I12" s="5" t="str">
+      <ns0:c r="B12" s="4">
+        <ns0:v>610</ns0:v>
+      </ns0:c>
+      <ns0:c r="C12" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D12" s="4">
+        <ns0:v>130</ns0:v>
+      </ns0:c>
+      <ns0:c r="E12" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="F12" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G12" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H12" s="4">
+        <ns0:v>220</ns0:v>
+      </ns0:c>
+      <ns0:c r="I12" s="5">
         <ns0:f t="shared" si="0"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J12" s="5" t="str">
+        <ns0:v>1340</ns0:v>
+      </ns0:c>
+      <ns0:c r="J12" s="5">
         <ns0:f t="shared" si="1"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K12" s="4"/>
-      <ns0:c r="L12" s="4"/>
-      <ns0:c r="M12" s="4"/>
-      <ns0:c r="N12" s="6"/>
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="K12" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L12" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M12" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N12" s="4" t="s">
+        <ns0:v>41</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="13" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A13" s="3">

</xml_diff>

<commit_message>
Update Day 8 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0302D5C8-EA0F-436E-A85F-12BE17B0D05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B7D623A-5FEF-4DFA-BC3B-3A9DF1C57A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1063,25 +1063,47 @@
       <ns0:c r="A13" s="3">
         <ns0:v>46254</ns0:v>
       </ns0:c>
-      <ns0:c r="B13" s="4"/>
-      <ns0:c r="C13" s="13"/>
-      <ns0:c r="D13" s="13"/>
-      <ns0:c r="E13" s="13"/>
-      <ns0:c r="F13" s="13"/>
-      <ns0:c r="G13" s="13"/>
-      <ns0:c r="H13" s="13"/>
-      <ns0:c r="I13" s="5" t="str">
+      <ns0:c r="B13" s="4">
+        <ns0:v>510</ns0:v>
+      </ns0:c>
+      <ns0:c r="C13" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D13" s="4">
+        <ns0:v>80</ns0:v>
+      </ns0:c>
+      <ns0:c r="E13" s="4">
+        <ns0:v>230</ns0:v>
+      </ns0:c>
+      <ns0:c r="F13" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="G13" s="4">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="H13" s="4">
+        <ns0:v>220</ns0:v>
+      </ns0:c>
+      <ns0:c r="I13" s="5">
         <ns0:f t="shared" ref="I13:I45" si="2">IF(COUNT(B13:F13,H13)&lt;6,"",SUM(B13:F13,H13))</ns0:f>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J13" s="5" t="str">
+        <ns0:v>1370</ns0:v>
+      </ns0:c>
+      <ns0:c r="J13" s="5">
         <ns0:f t="shared" ref="J13:J45" si="3">IF(I13="","",1440-I13)</ns0:f>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K13" s="4"/>
-      <ns0:c r="L13" s="4"/>
-      <ns0:c r="M13" s="4"/>
-      <ns0:c r="N13" s="6"/>
+        <ns0:v>70</ns0:v>
+      </ns0:c>
+      <ns0:c r="K13" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L13" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M13" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N13" s="4" t="s">
+        <ns0:v>36</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="14" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A14" s="3">

</xml_diff>

<commit_message>
Update Day 9 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B7D623A-5FEF-4DFA-BC3B-3A9DF1C57A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1453FE03-B288-43FB-AD52-C1470D15395F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1109,25 +1109,47 @@
       <ns0:c r="A14" s="3">
         <ns0:v>46255</ns0:v>
       </ns0:c>
-      <ns0:c r="B14" s="4"/>
-      <ns0:c r="C14" s="4"/>
-      <ns0:c r="D14" s="4"/>
-      <ns0:c r="E14" s="4"/>
-      <ns0:c r="F14" s="4"/>
-      <ns0:c r="G14" s="4"/>
-      <ns0:c r="H14" s="4"/>
-      <ns0:c r="I14" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J14" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K14" s="4"/>
-      <ns0:c r="L14" s="4"/>
-      <ns0:c r="M14" s="4"/>
-      <ns0:c r="N14" s="6"/>
+      <ns0:c r="B14" s="4">
+        <ns0:v>560</ns0:v>
+      </ns0:c>
+      <ns0:c r="C14" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D14" s="4">
+        <ns0:v>140</ns0:v>
+      </ns0:c>
+      <ns0:c r="E14" s="4">
+        <ns0:v>220</ns0:v>
+      </ns0:c>
+      <ns0:c r="F14" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G14" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H14" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I14" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1440</ns0:v>
+      </ns0:c>
+      <ns0:c r="J14" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K14" s="4" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="L14" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M14" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N14" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="15" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A15" s="3">
@@ -1905,7 +1927,7 @@
           <ns5:formula2>
             <ns6:f>0</ns6:f>
           </ns5:formula2>
-          <ns6:sqref>K6:K13</ns6:sqref>
+          <ns6:sqref>K6:K45</ns6:sqref>
         </ns5:dataValidation>
         <ns5:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Pick from list" error="Choose a value from the dropdown." ns2:uid="{00000000-0002-0000-0000-000003000000}">
           <ns5:formula1>
@@ -1914,7 +1936,7 @@
           <ns5:formula2>
             <ns6:f>0</ns6:f>
           </ns5:formula2>
-          <ns6:sqref>L6:L13</ns6:sqref>
+          <ns6:sqref>L6:L45</ns6:sqref>
         </ns5:dataValidation>
         <ns5:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Pick from list" error="Choose a value from the dropdown." ns2:uid="{00000000-0002-0000-0000-000004000000}">
           <ns5:formula1>
@@ -1923,7 +1945,7 @@
           <ns5:formula2>
             <ns6:f>0</ns6:f>
           </ns5:formula2>
-          <ns6:sqref>M6:M13</ns6:sqref>
+          <ns6:sqref>M6:M45</ns6:sqref>
         </ns5:dataValidation>
       </ns5:dataValidations>
     </ns0:ext>

</xml_diff>

<commit_message>
Update Day 10 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1453FE03-B288-43FB-AD52-C1470D15395F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98BDA298-4979-4752-9E34-F2010D6C55D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1155,25 +1155,47 @@
       <ns0:c r="A15" s="3">
         <ns0:v>46256</ns0:v>
       </ns0:c>
-      <ns0:c r="B15" s="4"/>
-      <ns0:c r="C15" s="13"/>
-      <ns0:c r="D15" s="13"/>
-      <ns0:c r="E15" s="13"/>
-      <ns0:c r="F15" s="13"/>
-      <ns0:c r="G15" s="13"/>
-      <ns0:c r="H15" s="13"/>
-      <ns0:c r="I15" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J15" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K15" s="4"/>
-      <ns0:c r="L15" s="4"/>
-      <ns0:c r="M15" s="4"/>
-      <ns0:c r="N15" s="6"/>
+      <ns0:c r="B15" s="4">
+        <ns0:v>530</ns0:v>
+      </ns0:c>
+      <ns0:c r="C15" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D15" s="4">
+        <ns0:v>190</ns0:v>
+      </ns0:c>
+      <ns0:c r="E15" s="4">
+        <ns0:v>340</ns0:v>
+      </ns0:c>
+      <ns0:c r="F15" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="G15" s="4">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="H15" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I15" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1430</ns0:v>
+      </ns0:c>
+      <ns0:c r="J15" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="K15" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L15" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M15" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N15" s="4" t="s">
+        <ns0:v>38</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="16" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A16" s="3">

</xml_diff>

<commit_message>
Update Day 11 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98BDA298-4979-4752-9E34-F2010D6C55D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86290B7A-99A4-4C6F-8F09-67E72529CBB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1201,25 +1201,47 @@
       <ns0:c r="A16" s="3">
         <ns0:v>46257</ns0:v>
       </ns0:c>
-      <ns0:c r="B16" s="4"/>
-      <ns0:c r="C16" s="13"/>
-      <ns0:c r="D16" s="13"/>
-      <ns0:c r="E16" s="13"/>
-      <ns0:c r="F16" s="13"/>
-      <ns0:c r="G16" s="13"/>
-      <ns0:c r="H16" s="13"/>
-      <ns0:c r="I16" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J16" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K16" s="4"/>
-      <ns0:c r="L16" s="4"/>
-      <ns0:c r="M16" s="4"/>
-      <ns0:c r="N16" s="6"/>
+      <ns0:c r="B16" s="4">
+        <ns0:v>520</ns0:v>
+      </ns0:c>
+      <ns0:c r="C16" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D16" s="4">
+        <ns0:v>110</ns0:v>
+      </ns0:c>
+      <ns0:c r="E16" s="4">
+        <ns0:v>400</ns0:v>
+      </ns0:c>
+      <ns0:c r="F16" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="G16" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="H16" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="I16" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1360</ns0:v>
+      </ns0:c>
+      <ns0:c r="J16" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>80</ns0:v>
+      </ns0:c>
+      <ns0:c r="K16" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L16" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M16" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N16" s="4" t="s">
+        <ns0:v>39</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="17" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A17" s="3">

</xml_diff>

<commit_message>
Update Day 12 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86290B7A-99A4-4C6F-8F09-67E72529CBB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FDA880-5614-41B2-A850-D1EF94633CE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1247,25 +1247,47 @@
       <ns0:c r="A17" s="3">
         <ns0:v>46258</ns0:v>
       </ns0:c>
-      <ns0:c r="B17" s="4"/>
-      <ns0:c r="C17" s="13"/>
-      <ns0:c r="D17" s="13"/>
-      <ns0:c r="E17" s="13"/>
-      <ns0:c r="F17" s="13"/>
-      <ns0:c r="G17" s="13"/>
-      <ns0:c r="H17" s="13"/>
-      <ns0:c r="I17" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J17" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K17" s="4"/>
-      <ns0:c r="L17" s="4"/>
-      <ns0:c r="M17" s="4"/>
-      <ns0:c r="N17" s="6"/>
+      <ns0:c r="B17" s="4">
+        <ns0:v>550</ns0:v>
+      </ns0:c>
+      <ns0:c r="C17" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D17" s="4">
+        <ns0:v>150</ns0:v>
+      </ns0:c>
+      <ns0:c r="E17" s="4">
+        <ns0:v>130</ns0:v>
+      </ns0:c>
+      <ns0:c r="F17" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G17" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H17" s="4">
+        <ns0:v>260</ns0:v>
+      </ns0:c>
+      <ns0:c r="I17" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1380</ns0:v>
+      </ns0:c>
+      <ns0:c r="J17" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>60</ns0:v>
+      </ns0:c>
+      <ns0:c r="K17" s="4" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="L17" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M17" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N17" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="18" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A18" s="3">

</xml_diff>

<commit_message>
Update Day 13 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FDA880-5614-41B2-A850-D1EF94633CE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{512EA0BA-FCB4-4709-B36C-5DCA929797A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1293,25 +1293,47 @@
       <ns0:c r="A18" s="3">
         <ns0:v>46259</ns0:v>
       </ns0:c>
-      <ns0:c r="B18" s="4"/>
-      <ns0:c r="C18" s="13"/>
-      <ns0:c r="D18" s="13"/>
-      <ns0:c r="E18" s="13"/>
-      <ns0:c r="F18" s="13"/>
-      <ns0:c r="G18" s="13"/>
-      <ns0:c r="H18" s="13"/>
-      <ns0:c r="I18" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J18" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K18" s="4"/>
-      <ns0:c r="L18" s="4"/>
-      <ns0:c r="M18" s="4"/>
-      <ns0:c r="N18" s="6"/>
+      <ns0:c r="B18" s="4">
+        <ns0:v>520</ns0:v>
+      </ns0:c>
+      <ns0:c r="C18" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D18" s="4">
+        <ns0:v>140</ns0:v>
+      </ns0:c>
+      <ns0:c r="E18" s="4">
+        <ns0:v>220</ns0:v>
+      </ns0:c>
+      <ns0:c r="F18" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G18" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H18" s="4">
+        <ns0:v>230</ns0:v>
+      </ns0:c>
+      <ns0:c r="I18" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1400</ns0:v>
+      </ns0:c>
+      <ns0:c r="J18" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="K18" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L18" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M18" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N18" s="4" t="s">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="19" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A19" s="3">

</xml_diff>

<commit_message>
Update Day 14 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{512EA0BA-FCB4-4709-B36C-5DCA929797A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F78ADE29-E8B6-4E0F-8002-530640ED04CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1339,25 +1339,47 @@
       <ns0:c r="A19" s="3">
         <ns0:v>46260</ns0:v>
       </ns0:c>
-      <ns0:c r="B19" s="4"/>
-      <ns0:c r="C19" s="13"/>
-      <ns0:c r="D19" s="13"/>
-      <ns0:c r="E19" s="13"/>
-      <ns0:c r="F19" s="13"/>
-      <ns0:c r="G19" s="13"/>
-      <ns0:c r="H19" s="13"/>
-      <ns0:c r="I19" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J19" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K19" s="4"/>
-      <ns0:c r="L19" s="4"/>
-      <ns0:c r="M19" s="4"/>
-      <ns0:c r="N19" s="6"/>
+      <ns0:c r="B19" s="4">
+        <ns0:v>600</ns0:v>
+      </ns0:c>
+      <ns0:c r="C19" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D19" s="4">
+        <ns0:v>110</ns0:v>
+      </ns0:c>
+      <ns0:c r="E19" s="4">
+        <ns0:v>150</ns0:v>
+      </ns0:c>
+      <ns0:c r="F19" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G19" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H19" s="4">
+        <ns0:v>260</ns0:v>
+      </ns0:c>
+      <ns0:c r="I19" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1400</ns0:v>
+      </ns0:c>
+      <ns0:c r="J19" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="K19" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L19" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M19" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N19" s="4" t="s">
+        <ns0:v>41</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="20" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A20" s="3">

</xml_diff>

<commit_message>
Update Day 15 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F78ADE29-E8B6-4E0F-8002-530640ED04CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{333CF77D-5EC8-43B9-ACE7-1D52E16CE6E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1385,25 +1385,47 @@
       <ns0:c r="A20" s="3">
         <ns0:v>46261</ns0:v>
       </ns0:c>
-      <ns0:c r="B20" s="4"/>
-      <ns0:c r="C20" s="13"/>
-      <ns0:c r="D20" s="13"/>
-      <ns0:c r="E20" s="13"/>
-      <ns0:c r="F20" s="13"/>
-      <ns0:c r="G20" s="13"/>
-      <ns0:c r="H20" s="13"/>
-      <ns0:c r="I20" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J20" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K20" s="4"/>
-      <ns0:c r="L20" s="4"/>
-      <ns0:c r="M20" s="4"/>
-      <ns0:c r="N20" s="6"/>
+      <ns0:c r="B20" s="4">
+        <ns0:v>550</ns0:v>
+      </ns0:c>
+      <ns0:c r="C20" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D20" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="E20" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="F20" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="G20" s="4">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="H20" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I20" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1420</ns0:v>
+      </ns0:c>
+      <ns0:c r="J20" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="K20" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L20" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M20" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N20" s="4" t="s">
+        <ns0:v>36</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="21" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A21" s="3">

</xml_diff>

<commit_message>
Update Day 16 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{333CF77D-5EC8-43B9-ACE7-1D52E16CE6E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E221B59-7DA2-4B6D-991E-15AE9A39E222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1431,25 +1431,47 @@
       <ns0:c r="A21" s="3">
         <ns0:v>46262</ns0:v>
       </ns0:c>
-      <ns0:c r="B21" s="4"/>
-      <ns0:c r="C21" s="13"/>
-      <ns0:c r="D21" s="13"/>
-      <ns0:c r="E21" s="13"/>
-      <ns0:c r="F21" s="13"/>
-      <ns0:c r="G21" s="13"/>
-      <ns0:c r="H21" s="13"/>
-      <ns0:c r="I21" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J21" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K21" s="4"/>
-      <ns0:c r="L21" s="4"/>
-      <ns0:c r="M21" s="4"/>
-      <ns0:c r="N21" s="6"/>
+      <ns0:c r="B21" s="4">
+        <ns0:v>560</ns0:v>
+      </ns0:c>
+      <ns0:c r="C21" s="4">
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="D21" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="E21" s="4">
+        <ns0:v>260</ns0:v>
+      </ns0:c>
+      <ns0:c r="F21" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G21" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H21" s="4">
+        <ns0:v>220</ns0:v>
+      </ns0:c>
+      <ns0:c r="I21" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1410</ns0:v>
+      </ns0:c>
+      <ns0:c r="J21" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="K21" s="4" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="L21" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M21" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N21" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="22" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A22" s="3">

</xml_diff>

<commit_message>
Update Day 17 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E221B59-7DA2-4B6D-991E-15AE9A39E222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E399741F-AE13-4EDA-8A77-E22AC32ACD0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1477,25 +1477,47 @@
       <ns0:c r="A22" s="3">
         <ns0:v>46263</ns0:v>
       </ns0:c>
-      <ns0:c r="B22" s="4"/>
-      <ns0:c r="C22" s="4"/>
-      <ns0:c r="D22" s="4"/>
-      <ns0:c r="E22" s="4"/>
-      <ns0:c r="F22" s="4"/>
-      <ns0:c r="G22" s="4"/>
-      <ns0:c r="H22" s="4"/>
-      <ns0:c r="I22" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J22" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K22" s="4"/>
-      <ns0:c r="L22" s="4"/>
-      <ns0:c r="M22" s="4"/>
-      <ns0:c r="N22" s="6"/>
+      <ns0:c r="B22" s="4">
+        <ns0:v>560</ns0:v>
+      </ns0:c>
+      <ns0:c r="C22" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D22" s="4">
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="E22" s="4">
+        <ns0:v>310</ns0:v>
+      </ns0:c>
+      <ns0:c r="F22" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="G22" s="4">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="H22" s="4">
+        <ns0:v>220</ns0:v>
+      </ns0:c>
+      <ns0:c r="I22" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1400</ns0:v>
+      </ns0:c>
+      <ns0:c r="J22" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="K22" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L22" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M22" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N22" s="4" t="s">
+        <ns0:v>38</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="23" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A23" s="3">

</xml_diff>

<commit_message>
Update Day 18 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E399741F-AE13-4EDA-8A77-E22AC32ACD0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98C4012-C668-493F-B7B0-E44D6EB235FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1523,25 +1523,47 @@
       <ns0:c r="A23" s="3">
         <ns0:v>46264</ns0:v>
       </ns0:c>
-      <ns0:c r="B23" s="4"/>
-      <ns0:c r="C23" s="13"/>
-      <ns0:c r="D23" s="13"/>
-      <ns0:c r="E23" s="13"/>
-      <ns0:c r="F23" s="13"/>
-      <ns0:c r="G23" s="13"/>
-      <ns0:c r="H23" s="13"/>
-      <ns0:c r="I23" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J23" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K23" s="4"/>
-      <ns0:c r="L23" s="4"/>
-      <ns0:c r="M23" s="4"/>
-      <ns0:c r="N23" s="6"/>
+      <ns0:c r="B23" s="4">
+        <ns0:v>520</ns0:v>
+      </ns0:c>
+      <ns0:c r="C23" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D23" s="4">
+        <ns0:v>150</ns0:v>
+      </ns0:c>
+      <ns0:c r="E23" s="4">
+        <ns0:v>420</ns0:v>
+      </ns0:c>
+      <ns0:c r="F23" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="G23" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="H23" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="I23" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1430</ns0:v>
+      </ns0:c>
+      <ns0:c r="J23" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="K23" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L23" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M23" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N23" s="4" t="s">
+        <ns0:v>39</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="24" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A24" s="3">

</xml_diff>

<commit_message>
Update Day 19 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98C4012-C668-493F-B7B0-E44D6EB235FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0011BE-A3D2-4443-A236-20DCD35FA690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1569,25 +1569,47 @@
       <ns0:c r="A24" s="3">
         <ns0:v>46265</ns0:v>
       </ns0:c>
-      <ns0:c r="B24" s="4"/>
-      <ns0:c r="C24" s="13"/>
-      <ns0:c r="D24" s="13"/>
-      <ns0:c r="E24" s="13"/>
-      <ns0:c r="F24" s="13"/>
-      <ns0:c r="G24" s="13"/>
-      <ns0:c r="H24" s="13"/>
-      <ns0:c r="I24" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J24" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K24" s="4"/>
-      <ns0:c r="L24" s="4"/>
-      <ns0:c r="M24" s="4"/>
-      <ns0:c r="N24" s="6"/>
+      <ns0:c r="B24" s="4">
+        <ns0:v>560</ns0:v>
+      </ns0:c>
+      <ns0:c r="C24" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D24" s="4">
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="E24" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="F24" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G24" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H24" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="I24" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1400</ns0:v>
+      </ns0:c>
+      <ns0:c r="J24" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="K24" s="4" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="L24" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M24" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N24" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="25" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A25" s="3">

</xml_diff>

<commit_message>
Update Day 20 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0011BE-A3D2-4443-A236-20DCD35FA690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C71CD8-2509-436F-8770-6D5CACBEDD7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1615,25 +1615,47 @@
       <ns0:c r="A25" s="3">
         <ns0:v>46266</ns0:v>
       </ns0:c>
-      <ns0:c r="B25" s="4"/>
-      <ns0:c r="C25" s="13"/>
-      <ns0:c r="D25" s="13"/>
-      <ns0:c r="E25" s="13"/>
-      <ns0:c r="F25" s="13"/>
-      <ns0:c r="G25" s="13"/>
-      <ns0:c r="H25" s="13"/>
-      <ns0:c r="I25" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J25" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K25" s="4"/>
-      <ns0:c r="L25" s="4"/>
-      <ns0:c r="M25" s="4"/>
-      <ns0:c r="N25" s="6"/>
+      <ns0:c r="B25" s="4">
+        <ns0:v>520</ns0:v>
+      </ns0:c>
+      <ns0:c r="C25" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D25" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="E25" s="4">
+        <ns0:v>220</ns0:v>
+      </ns0:c>
+      <ns0:c r="F25" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G25" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H25" s="4">
+        <ns0:v>260</ns0:v>
+      </ns0:c>
+      <ns0:c r="I25" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1380</ns0:v>
+      </ns0:c>
+      <ns0:c r="J25" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>60</ns0:v>
+      </ns0:c>
+      <ns0:c r="K25" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L25" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M25" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N25" s="4" t="s">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="26" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A26" s="3">

</xml_diff>

<commit_message>
Update Day 21 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C71CD8-2509-436F-8770-6D5CACBEDD7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD492FB-2232-4330-9792-925160D065D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1661,25 +1661,47 @@
       <ns0:c r="A26" s="3">
         <ns0:v>46267</ns0:v>
       </ns0:c>
-      <ns0:c r="B26" s="4"/>
-      <ns0:c r="C26" s="13"/>
-      <ns0:c r="D26" s="13"/>
-      <ns0:c r="E26" s="13"/>
-      <ns0:c r="F26" s="13"/>
-      <ns0:c r="G26" s="13"/>
-      <ns0:c r="H26" s="13"/>
-      <ns0:c r="I26" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J26" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K26" s="4"/>
-      <ns0:c r="L26" s="4"/>
-      <ns0:c r="M26" s="4"/>
-      <ns0:c r="N26" s="6"/>
+      <ns0:c r="B26" s="4">
+        <ns0:v>600</ns0:v>
+      </ns0:c>
+      <ns0:c r="C26" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D26" s="4">
+        <ns0:v>140</ns0:v>
+      </ns0:c>
+      <ns0:c r="E26" s="4">
+        <ns0:v>130</ns0:v>
+      </ns0:c>
+      <ns0:c r="F26" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G26" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H26" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="I26" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1400</ns0:v>
+      </ns0:c>
+      <ns0:c r="J26" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="K26" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L26" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M26" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N26" s="4" t="s">
+        <ns0:v>41</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="27" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A27" s="3">

</xml_diff>

<commit_message>
Update Day 22 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD492FB-2232-4330-9792-925160D065D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C4FB15B-FCEF-4E77-A93B-B648B55D3A37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1707,25 +1707,47 @@
       <ns0:c r="A27" s="3">
         <ns0:v>46268</ns0:v>
       </ns0:c>
-      <ns0:c r="B27" s="4"/>
-      <ns0:c r="C27" s="13"/>
-      <ns0:c r="D27" s="13"/>
-      <ns0:c r="E27" s="13"/>
-      <ns0:c r="F27" s="13"/>
-      <ns0:c r="G27" s="13"/>
-      <ns0:c r="H27" s="13"/>
-      <ns0:c r="I27" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J27" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K27" s="4"/>
-      <ns0:c r="L27" s="4"/>
-      <ns0:c r="M27" s="4"/>
-      <ns0:c r="N27" s="6"/>
+      <ns0:c r="B27" s="4">
+        <ns0:v>570</ns0:v>
+      </ns0:c>
+      <ns0:c r="C27" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D27" s="4">
+        <ns0:v>60</ns0:v>
+      </ns0:c>
+      <ns0:c r="E27" s="4">
+        <ns0:v>230</ns0:v>
+      </ns0:c>
+      <ns0:c r="F27" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="G27" s="4">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="H27" s="4">
+        <ns0:v>230</ns0:v>
+      </ns0:c>
+      <ns0:c r="I27" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1430</ns0:v>
+      </ns0:c>
+      <ns0:c r="J27" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="K27" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L27" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M27" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N27" s="4" t="s">
+        <ns0:v>36</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="28" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A28" s="3">

</xml_diff>

<commit_message>
Update Day 23 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C4FB15B-FCEF-4E77-A93B-B648B55D3A37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{063B3B05-A312-4089-9300-AC9169CEAC1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1753,25 +1753,47 @@
       <ns0:c r="A28" s="3">
         <ns0:v>46269</ns0:v>
       </ns0:c>
-      <ns0:c r="B28" s="4"/>
-      <ns0:c r="C28" s="13"/>
-      <ns0:c r="D28" s="13"/>
-      <ns0:c r="E28" s="13"/>
-      <ns0:c r="F28" s="13"/>
-      <ns0:c r="G28" s="13"/>
-      <ns0:c r="H28" s="13"/>
-      <ns0:c r="I28" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J28" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K28" s="4"/>
-      <ns0:c r="L28" s="4"/>
-      <ns0:c r="M28" s="4"/>
-      <ns0:c r="N28" s="6"/>
+      <ns0:c r="B28" s="4">
+        <ns0:v>520</ns0:v>
+      </ns0:c>
+      <ns0:c r="C28" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D28" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="E28" s="4">
+        <ns0:v>220</ns0:v>
+      </ns0:c>
+      <ns0:c r="F28" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G28" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H28" s="4">
+        <ns0:v>220</ns0:v>
+      </ns0:c>
+      <ns0:c r="I28" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1370</ns0:v>
+      </ns0:c>
+      <ns0:c r="J28" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>70</ns0:v>
+      </ns0:c>
+      <ns0:c r="K28" s="4" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="L28" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M28" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N28" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="29" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A29" s="3">

</xml_diff>

<commit_message>
Update Day 24 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{063B3B05-A312-4089-9300-AC9169CEAC1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCFE432D-E6CC-4A9B-9AEF-19658CEEB64A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1799,25 +1799,47 @@
       <ns0:c r="A29" s="3">
         <ns0:v>46270</ns0:v>
       </ns0:c>
-      <ns0:c r="B29" s="4"/>
-      <ns0:c r="C29" s="13"/>
-      <ns0:c r="D29" s="13"/>
-      <ns0:c r="E29" s="13"/>
-      <ns0:c r="F29" s="13"/>
-      <ns0:c r="G29" s="13"/>
-      <ns0:c r="H29" s="13"/>
-      <ns0:c r="I29" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J29" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K29" s="4"/>
-      <ns0:c r="L29" s="4"/>
-      <ns0:c r="M29" s="4"/>
-      <ns0:c r="N29" s="6"/>
+      <ns0:c r="B29" s="4">
+        <ns0:v>560</ns0:v>
+      </ns0:c>
+      <ns0:c r="C29" s="4">
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="D29" s="4">
+        <ns0:v>160</ns0:v>
+      </ns0:c>
+      <ns0:c r="E29" s="4">
+        <ns0:v>330</ns0:v>
+      </ns0:c>
+      <ns0:c r="F29" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="G29" s="4">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="H29" s="4">
+        <ns0:v>230</ns0:v>
+      </ns0:c>
+      <ns0:c r="I29" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1400</ns0:v>
+      </ns0:c>
+      <ns0:c r="J29" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="K29" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L29" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M29" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N29" s="4" t="s">
+        <ns0:v>38</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="30" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A30" s="3">

</xml_diff>

<commit_message>
Update Day 25 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCFE432D-E6CC-4A9B-9AEF-19658CEEB64A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC59F79-EFAF-4D5D-8336-B992E225EB7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1845,25 +1845,47 @@
       <ns0:c r="A30" s="3">
         <ns0:v>46271</ns0:v>
       </ns0:c>
-      <ns0:c r="B30" s="4"/>
-      <ns0:c r="C30" s="4"/>
-      <ns0:c r="D30" s="4"/>
-      <ns0:c r="E30" s="4"/>
-      <ns0:c r="F30" s="4"/>
-      <ns0:c r="G30" s="4"/>
-      <ns0:c r="H30" s="4"/>
-      <ns0:c r="I30" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J30" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K30" s="4"/>
-      <ns0:c r="L30" s="4"/>
-      <ns0:c r="M30" s="4"/>
-      <ns0:c r="N30" s="6"/>
+      <ns0:c r="B30" s="4">
+        <ns0:v>560</ns0:v>
+      </ns0:c>
+      <ns0:c r="C30" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D30" s="4">
+        <ns0:v>130</ns0:v>
+      </ns0:c>
+      <ns0:c r="E30" s="4">
+        <ns0:v>390</ns0:v>
+      </ns0:c>
+      <ns0:c r="F30" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="G30" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="H30" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="I30" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1410</ns0:v>
+      </ns0:c>
+      <ns0:c r="J30" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="K30" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L30" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M30" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N30" s="4" t="s">
+        <ns0:v>39</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="31" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A31" s="3">

</xml_diff>

<commit_message>
Update Day 26 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC59F79-EFAF-4D5D-8336-B992E225EB7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD353D68-699D-4244-B75A-89320FD9872C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1891,25 +1891,47 @@
       <ns0:c r="A31" s="3">
         <ns0:v>46272</ns0:v>
       </ns0:c>
-      <ns0:c r="B31" s="4"/>
-      <ns0:c r="C31" s="13"/>
-      <ns0:c r="D31" s="13"/>
-      <ns0:c r="E31" s="13"/>
-      <ns0:c r="F31" s="13"/>
-      <ns0:c r="G31" s="13"/>
-      <ns0:c r="H31" s="13"/>
-      <ns0:c r="I31" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J31" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K31" s="4"/>
-      <ns0:c r="L31" s="4"/>
-      <ns0:c r="M31" s="4"/>
-      <ns0:c r="N31" s="6"/>
+      <ns0:c r="B31" s="4">
+        <ns0:v>530</ns0:v>
+      </ns0:c>
+      <ns0:c r="C31" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D31" s="4">
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="E31" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="F31" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G31" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H31" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I31" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1360</ns0:v>
+      </ns0:c>
+      <ns0:c r="J31" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>80</ns0:v>
+      </ns0:c>
+      <ns0:c r="K31" s="4" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="L31" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M31" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N31" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="32" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A32" s="3">

</xml_diff>

<commit_message>
Update Day 27 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD353D68-699D-4244-B75A-89320FD9872C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57C4D5C9-8CB7-4B72-85D4-A03CE4545484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1937,25 +1937,47 @@
       <ns0:c r="A32" s="3">
         <ns0:v>46273</ns0:v>
       </ns0:c>
-      <ns0:c r="B32" s="4"/>
-      <ns0:c r="C32" s="13"/>
-      <ns0:c r="D32" s="13"/>
-      <ns0:c r="E32" s="13"/>
-      <ns0:c r="F32" s="13"/>
-      <ns0:c r="G32" s="13"/>
-      <ns0:c r="H32" s="13"/>
-      <ns0:c r="I32" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J32" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K32" s="4"/>
-      <ns0:c r="L32" s="4"/>
-      <ns0:c r="M32" s="4"/>
-      <ns0:c r="N32" s="6"/>
+      <ns0:c r="B32" s="4">
+        <ns0:v>540</ns0:v>
+      </ns0:c>
+      <ns0:c r="C32" s="4">
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="D32" s="4">
+        <ns0:v>130</ns0:v>
+      </ns0:c>
+      <ns0:c r="E32" s="4">
+        <ns0:v>260</ns0:v>
+      </ns0:c>
+      <ns0:c r="F32" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G32" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H32" s="4">
+        <ns0:v>230</ns0:v>
+      </ns0:c>
+      <ns0:c r="I32" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1430</ns0:v>
+      </ns0:c>
+      <ns0:c r="J32" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="K32" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L32" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M32" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N32" s="4" t="s">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="33" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A33" s="3">

</xml_diff>

<commit_message>
Update Day 28 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57C4D5C9-8CB7-4B72-85D4-A03CE4545484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F8A8745-ACA1-4649-B85E-7B3D17A3F81F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -1983,25 +1983,47 @@
       <ns0:c r="A33" s="3">
         <ns0:v>46274</ns0:v>
       </ns0:c>
-      <ns0:c r="B33" s="4"/>
-      <ns0:c r="C33" s="13"/>
-      <ns0:c r="D33" s="13"/>
-      <ns0:c r="E33" s="13"/>
-      <ns0:c r="F33" s="13"/>
-      <ns0:c r="G33" s="13"/>
-      <ns0:c r="H33" s="13"/>
-      <ns0:c r="I33" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J33" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K33" s="4"/>
-      <ns0:c r="L33" s="4"/>
-      <ns0:c r="M33" s="4"/>
-      <ns0:c r="N33" s="6"/>
+      <ns0:c r="B33" s="4">
+        <ns0:v>610</ns0:v>
+      </ns0:c>
+      <ns0:c r="C33" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D33" s="4">
+        <ns0:v>140</ns0:v>
+      </ns0:c>
+      <ns0:c r="E33" s="4">
+        <ns0:v>110</ns0:v>
+      </ns0:c>
+      <ns0:c r="F33" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G33" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H33" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I33" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1390</ns0:v>
+      </ns0:c>
+      <ns0:c r="J33" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>50</ns0:v>
+      </ns0:c>
+      <ns0:c r="K33" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L33" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M33" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N33" s="4" t="s">
+        <ns0:v>41</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="34" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A34" s="3">

</xml_diff>

<commit_message>
Update Day 29 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F8A8745-ACA1-4649-B85E-7B3D17A3F81F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51140860-A4F8-4369-B3D8-2153E4C2BF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -2029,25 +2029,47 @@
       <ns0:c r="A34" s="3">
         <ns0:v>46275</ns0:v>
       </ns0:c>
-      <ns0:c r="B34" s="4"/>
-      <ns0:c r="C34" s="13"/>
-      <ns0:c r="D34" s="13"/>
-      <ns0:c r="E34" s="13"/>
-      <ns0:c r="F34" s="13"/>
-      <ns0:c r="G34" s="13"/>
-      <ns0:c r="H34" s="13"/>
-      <ns0:c r="I34" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J34" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K34" s="4"/>
-      <ns0:c r="L34" s="4"/>
-      <ns0:c r="M34" s="4"/>
-      <ns0:c r="N34" s="6"/>
+      <ns0:c r="B34" s="4">
+        <ns0:v>520</ns0:v>
+      </ns0:c>
+      <ns0:c r="C34" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D34" s="4">
+        <ns0:v>60</ns0:v>
+      </ns0:c>
+      <ns0:c r="E34" s="4">
+        <ns0:v>220</ns0:v>
+      </ns0:c>
+      <ns0:c r="F34" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="G34" s="4">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="H34" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="I34" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1380</ns0:v>
+      </ns0:c>
+      <ns0:c r="J34" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>60</ns0:v>
+      </ns0:c>
+      <ns0:c r="K34" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L34" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M34" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N34" s="4" t="s">
+        <ns0:v>36</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="35" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A35" s="3">

</xml_diff>

<commit_message>
Update Day 30 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51140860-A4F8-4369-B3D8-2153E4C2BF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E81595-F733-4397-B00A-7D5B8073A49F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -2075,25 +2075,47 @@
       <ns0:c r="A35" s="3">
         <ns0:v>46276</ns0:v>
       </ns0:c>
-      <ns0:c r="B35" s="4"/>
-      <ns0:c r="C35" s="13"/>
-      <ns0:c r="D35" s="13"/>
-      <ns0:c r="E35" s="13"/>
-      <ns0:c r="F35" s="13"/>
-      <ns0:c r="G35" s="13"/>
-      <ns0:c r="H35" s="13"/>
-      <ns0:c r="I35" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J35" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K35" s="4"/>
-      <ns0:c r="L35" s="4"/>
-      <ns0:c r="M35" s="4"/>
-      <ns0:c r="N35" s="6"/>
+      <ns0:c r="B35" s="4">
+        <ns0:v>510</ns0:v>
+      </ns0:c>
+      <ns0:c r="C35" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D35" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="E35" s="4">
+        <ns0:v>260</ns0:v>
+      </ns0:c>
+      <ns0:c r="F35" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G35" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H35" s="4">
+        <ns0:v>230</ns0:v>
+      </ns0:c>
+      <ns0:c r="I35" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1400</ns0:v>
+      </ns0:c>
+      <ns0:c r="J35" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="K35" s="4" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="L35" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M35" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N35" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="36" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A36" s="3">

</xml_diff>

<commit_message>
Update Day 31 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E81595-F733-4397-B00A-7D5B8073A49F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7ABBB9-C19F-479D-80D0-58E94310C2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -2121,25 +2121,47 @@
       <ns0:c r="A36" s="3">
         <ns0:v>46277</ns0:v>
       </ns0:c>
-      <ns0:c r="B36" s="4"/>
-      <ns0:c r="C36" s="13"/>
-      <ns0:c r="D36" s="13"/>
-      <ns0:c r="E36" s="13"/>
-      <ns0:c r="F36" s="13"/>
-      <ns0:c r="G36" s="13"/>
-      <ns0:c r="H36" s="13"/>
-      <ns0:c r="I36" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J36" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K36" s="4"/>
-      <ns0:c r="L36" s="4"/>
-      <ns0:c r="M36" s="4"/>
-      <ns0:c r="N36" s="6"/>
+      <ns0:c r="B36" s="4">
+        <ns0:v>540</ns0:v>
+      </ns0:c>
+      <ns0:c r="C36" s="4">
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="D36" s="4">
+        <ns0:v>200</ns0:v>
+      </ns0:c>
+      <ns0:c r="E36" s="4">
+        <ns0:v>330</ns0:v>
+      </ns0:c>
+      <ns0:c r="F36" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="G36" s="4">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="H36" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I36" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1430</ns0:v>
+      </ns0:c>
+      <ns0:c r="J36" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="K36" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L36" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M36" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N36" s="4" t="s">
+        <ns0:v>38</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="37" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A37" s="3">

</xml_diff>

<commit_message>
Update Day 32 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7ABBB9-C19F-479D-80D0-58E94310C2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5625D014-9B94-4327-9AEB-2F7A4CF93160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -2167,25 +2167,47 @@
       <ns0:c r="A37" s="3">
         <ns0:v>46278</ns0:v>
       </ns0:c>
-      <ns0:c r="B37" s="4"/>
-      <ns0:c r="C37" s="13"/>
-      <ns0:c r="D37" s="13"/>
-      <ns0:c r="E37" s="13"/>
-      <ns0:c r="F37" s="13"/>
-      <ns0:c r="G37" s="13"/>
-      <ns0:c r="H37" s="13"/>
-      <ns0:c r="I37" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J37" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K37" s="4"/>
-      <ns0:c r="L37" s="4"/>
-      <ns0:c r="M37" s="4"/>
-      <ns0:c r="N37" s="6"/>
+      <ns0:c r="B37" s="4">
+        <ns0:v>560</ns0:v>
+      </ns0:c>
+      <ns0:c r="C37" s="4">
+        <ns0:v>40</ns0:v>
+      </ns0:c>
+      <ns0:c r="D37" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="E37" s="4">
+        <ns0:v>430</ns0:v>
+      </ns0:c>
+      <ns0:c r="F37" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="G37" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="H37" s="4">
+        <ns0:v>290</ns0:v>
+      </ns0:c>
+      <ns0:c r="I37" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1440</ns0:v>
+      </ns0:c>
+      <ns0:c r="J37" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K37" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L37" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M37" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N37" s="4" t="s">
+        <ns0:v>39</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="38" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A38" s="3">

</xml_diff>

<commit_message>
Update Day 33 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5625D014-9B94-4327-9AEB-2F7A4CF93160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEF93741-DB67-4BCE-A808-88CE18A1DB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -2213,25 +2213,47 @@
       <ns0:c r="A38" s="3">
         <ns0:v>46279</ns0:v>
       </ns0:c>
-      <ns0:c r="B38" s="4"/>
-      <ns0:c r="C38" s="4"/>
-      <ns0:c r="D38" s="4"/>
-      <ns0:c r="E38" s="4"/>
-      <ns0:c r="F38" s="4"/>
-      <ns0:c r="G38" s="4"/>
-      <ns0:c r="H38" s="4"/>
-      <ns0:c r="I38" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J38" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K38" s="4"/>
-      <ns0:c r="L38" s="4"/>
-      <ns0:c r="M38" s="4"/>
-      <ns0:c r="N38" s="6"/>
+      <ns0:c r="B38" s="4">
+        <ns0:v>520</ns0:v>
+      </ns0:c>
+      <ns0:c r="C38" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D38" s="4">
+        <ns0:v>200</ns0:v>
+      </ns0:c>
+      <ns0:c r="E38" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="F38" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G38" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H38" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="I38" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1350</ns0:v>
+      </ns0:c>
+      <ns0:c r="J38" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>90</ns0:v>
+      </ns0:c>
+      <ns0:c r="K38" s="4" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="L38" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M38" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N38" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="39" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A39" s="3">

</xml_diff>

<commit_message>
Update Day 34 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEF93741-DB67-4BCE-A808-88CE18A1DB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72482BE5-077C-4471-8BF4-FC9ACE6317AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="42">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -2259,25 +2259,47 @@
       <ns0:c r="A39" s="3">
         <ns0:v>46280</ns0:v>
       </ns0:c>
-      <ns0:c r="B39" s="4"/>
-      <ns0:c r="C39" s="13"/>
-      <ns0:c r="D39" s="13"/>
-      <ns0:c r="E39" s="13"/>
-      <ns0:c r="F39" s="13"/>
-      <ns0:c r="G39" s="13"/>
-      <ns0:c r="H39" s="13"/>
-      <ns0:c r="I39" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J39" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K39" s="4"/>
-      <ns0:c r="L39" s="4"/>
-      <ns0:c r="M39" s="4"/>
-      <ns0:c r="N39" s="6"/>
+      <ns0:c r="B39" s="4">
+        <ns0:v>540</ns0:v>
+      </ns0:c>
+      <ns0:c r="C39" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D39" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="E39" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="F39" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G39" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H39" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I39" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1420</ns0:v>
+      </ns0:c>
+      <ns0:c r="J39" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="K39" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L39" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M39" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N39" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="40" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A40" s="3">

</xml_diff>

<commit_message>
Update Day 35 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72482BE5-077C-4471-8BF4-FC9ACE6317AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA348B4-D195-454E-B1E3-F30024E62196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="43">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -183,6 +183,9 @@
   </si>
   <si>
     <t>Steady progress</t>
+  </si>
+  <si>
+    <t>Full lecture</t>
   </si>
 </sst>
 </file>
@@ -2305,25 +2308,47 @@
       <ns0:c r="A40" s="3">
         <ns0:v>46281</ns0:v>
       </ns0:c>
-      <ns0:c r="B40" s="4"/>
-      <ns0:c r="C40" s="13"/>
-      <ns0:c r="D40" s="13"/>
-      <ns0:c r="E40" s="13"/>
-      <ns0:c r="F40" s="13"/>
-      <ns0:c r="G40" s="13"/>
-      <ns0:c r="H40" s="13"/>
-      <ns0:c r="I40" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J40" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K40" s="4"/>
-      <ns0:c r="L40" s="4"/>
-      <ns0:c r="M40" s="4"/>
-      <ns0:c r="N40" s="6"/>
+      <ns0:c r="B40" s="4">
+        <ns0:v>600</ns0:v>
+      </ns0:c>
+      <ns0:c r="C40" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D40" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="E40" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="F40" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G40" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H40" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I40" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1360</ns0:v>
+      </ns0:c>
+      <ns0:c r="J40" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>80</ns0:v>
+      </ns0:c>
+      <ns0:c r="K40" s="4" t="s">
+        <ns0:v>31</ns0:v>
+      </ns0:c>
+      <ns0:c r="L40" s="4" t="s">
+        <ns0:v>32</ns0:v>
+      </ns0:c>
+      <ns0:c r="M40" s="4" t="s">
+        <ns0:v>31</ns0:v>
+      </ns0:c>
+      <ns0:c r="N40" s="4" t="s">
+        <ns0:v>42</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="41" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A41" s="3">

</xml_diff>

<commit_message>
Update Day 36 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA348B4-D195-454E-B1E3-F30024E62196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B19E14E-806A-43E2-9F1E-731FB2DBE8EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="44">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -186,6 +186,9 @@
   </si>
   <si>
     <t>Full lecture</t>
+  </si>
+  <si>
+    <t>Practicles and less study</t>
   </si>
 </sst>
 </file>
@@ -2354,25 +2357,47 @@
       <ns0:c r="A41" s="3">
         <ns0:v>46282</ns0:v>
       </ns0:c>
-      <ns0:c r="B41" s="4"/>
-      <ns0:c r="C41" s="13"/>
-      <ns0:c r="D41" s="13"/>
-      <ns0:c r="E41" s="13"/>
-      <ns0:c r="F41" s="13"/>
-      <ns0:c r="G41" s="13"/>
-      <ns0:c r="H41" s="13"/>
-      <ns0:c r="I41" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J41" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K41" s="4"/>
-      <ns0:c r="L41" s="4"/>
-      <ns0:c r="M41" s="4"/>
-      <ns0:c r="N41" s="6"/>
+      <ns0:c r="B41" s="4">
+        <ns0:v>540</ns0:v>
+      </ns0:c>
+      <ns0:c r="C41" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D41" s="4">
+        <ns0:v>60</ns0:v>
+      </ns0:c>
+      <ns0:c r="E41" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="F41" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="G41" s="4">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="H41" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I41" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1410</ns0:v>
+      </ns0:c>
+      <ns0:c r="J41" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="K41" s="4" t="s">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="L41" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M41" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N41" s="4" t="s">
+        <ns0:v>43</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="42" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A42" s="3">

</xml_diff>

<commit_message>
Update Day 37 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B19E14E-806A-43E2-9F1E-731FB2DBE8EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3D4A4D-9E3C-461D-9214-2AFE0BCD464F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="44">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -2403,25 +2403,47 @@
       <ns0:c r="A42" s="3">
         <ns0:v>46283</ns0:v>
       </ns0:c>
-      <ns0:c r="B42" s="4"/>
-      <ns0:c r="C42" s="13"/>
-      <ns0:c r="D42" s="13"/>
-      <ns0:c r="E42" s="13"/>
-      <ns0:c r="F42" s="13"/>
-      <ns0:c r="G42" s="13"/>
-      <ns0:c r="H42" s="13"/>
-      <ns0:c r="I42" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J42" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K42" s="4"/>
-      <ns0:c r="L42" s="4"/>
-      <ns0:c r="M42" s="4"/>
-      <ns0:c r="N42" s="6"/>
+      <ns0:c r="B42" s="4">
+        <ns0:v>540</ns0:v>
+      </ns0:c>
+      <ns0:c r="C42" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D42" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="E42" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="F42" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G42" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H42" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I42" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1420</ns0:v>
+      </ns0:c>
+      <ns0:c r="J42" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>20</ns0:v>
+      </ns0:c>
+      <ns0:c r="K42" s="4" t="s">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="L42" s="4" t="s">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="M42" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N42" s="4" t="s">
+        <ns0:v>37</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="43" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A43" s="3">

</xml_diff>

<commit_message>
Update Day 38 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3D4A4D-9E3C-461D-9214-2AFE0BCD464F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B08DA6C7-D5CD-4432-9F15-0DD1711E1EAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="45">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -189,6 +189,9 @@
   </si>
   <si>
     <t>Practicles and less study</t>
+  </si>
+  <si>
+    <t>Focus on project and notes</t>
   </si>
 </sst>
 </file>
@@ -2449,37 +2452,59 @@
       <ns0:c r="A43" s="3">
         <ns0:v>46284</ns0:v>
       </ns0:c>
-      <ns0:c r="B43" s="4"/>
-      <ns0:c r="C43" s="13"/>
-      <ns0:c r="D43" s="13"/>
-      <ns0:c r="E43" s="13"/>
-      <ns0:c r="F43" s="13"/>
-      <ns0:c r="G43" s="13"/>
-      <ns0:c r="H43" s="13"/>
-      <ns0:c r="I43" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J43" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K43" s="4"/>
-      <ns0:c r="L43" s="4"/>
-      <ns0:c r="M43" s="4"/>
-      <ns0:c r="N43" s="6"/>
+      <ns0:c r="B43" s="4">
+        <ns0:v>540</ns0:v>
+      </ns0:c>
+      <ns0:c r="C43" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D43" s="4">
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="E43" s="4">
+        <ns0:v>320</ns0:v>
+      </ns0:c>
+      <ns0:c r="F43" s="4">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="G43" s="4">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="H43" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I43" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1410</ns0:v>
+      </ns0:c>
+      <ns0:c r="J43" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="K43" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L43" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M43" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N43" s="4" t="s">
+        <ns0:v>44</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="44" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A44" s="3">
         <ns0:v>46285</ns0:v>
       </ns0:c>
       <ns0:c r="B44" s="4"/>
-      <ns0:c r="C44" s="13"/>
-      <ns0:c r="D44" s="13"/>
-      <ns0:c r="E44" s="13"/>
-      <ns0:c r="F44" s="13"/>
-      <ns0:c r="G44" s="13"/>
-      <ns0:c r="H44" s="13"/>
+      <ns0:c r="C44" s="4"/>
+      <ns0:c r="D44" s="4"/>
+      <ns0:c r="E44" s="4"/>
+      <ns0:c r="F44" s="4"/>
+      <ns0:c r="G44" s="4"/>
+      <ns0:c r="H44" s="4"/>
       <ns0:c r="I44" s="5" t="str">
         <ns0:f t="shared" si="2"/>
         <ns0:v/>
@@ -2491,7 +2516,7 @@
       <ns0:c r="K44" s="4"/>
       <ns0:c r="L44" s="4"/>
       <ns0:c r="M44" s="4"/>
-      <ns0:c r="N44" s="6"/>
+      <ns0:c r="N44" s="4"/>
     </ns0:row>
     <ns0:row r="45" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A45" s="3">

</xml_diff>

<commit_message>
Update Day 39 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B08DA6C7-D5CD-4432-9F15-0DD1711E1EAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2469921D-021A-4EA5-8E2A-2758B21DD0C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2499,12 +2499,12 @@
         <ns0:v>46285</ns0:v>
       </ns0:c>
       <ns0:c r="B44" s="4"/>
-      <ns0:c r="C44" s="4"/>
-      <ns0:c r="D44" s="4"/>
-      <ns0:c r="E44" s="4"/>
-      <ns0:c r="F44" s="4"/>
-      <ns0:c r="G44" s="4"/>
-      <ns0:c r="H44" s="4"/>
+      <ns0:c r="C44" s="13"/>
+      <ns0:c r="D44" s="13"/>
+      <ns0:c r="E44" s="13"/>
+      <ns0:c r="F44" s="13"/>
+      <ns0:c r="G44" s="13"/>
+      <ns0:c r="H44" s="13"/>
       <ns0:c r="I44" s="5" t="str">
         <ns0:f t="shared" si="2"/>
         <ns0:v/>
@@ -2516,7 +2516,7 @@
       <ns0:c r="K44" s="4"/>
       <ns0:c r="L44" s="4"/>
       <ns0:c r="M44" s="4"/>
-      <ns0:c r="N44" s="4"/>
+      <ns0:c r="N44" s="6"/>
     </ns0:row>
     <ns0:row r="45" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A45" s="3">

</xml_diff>

<commit_message>
Update Day 40 activity data
</commit_message>
<xml_diff>
--- a/data/12617525.xlsx
+++ b/data/12617525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\codeLabPraveen\own\program\python\prj\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2469921D-021A-4EA5-8E2A-2758B21DD0C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01EBE37D-D2FC-4822-9F49-AE1E88EA316E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="47">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -192,6 +192,12 @@
   </si>
   <si>
     <t>Focus on project and notes</t>
+  </si>
+  <si>
+    <t>Focus on project and revision</t>
+  </si>
+  <si>
+    <t>Making notes</t>
   </si>
 </sst>
 </file>
@@ -277,7 +283,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -313,24 +319,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFBFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFBFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFBFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -345,9 +338,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -356,9 +346,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -658,44 +645,44 @@
   </ns0:cols>
   <ns0:sheetData>
     <ns0:row r="1" spans="1:14" ht="40.200000000000003" customHeight="1" ns3:dyDescent="0.3">
-      <ns0:c r="A1" s="14" t="s">
+      <ns0:c r="A1" s="12" t="s">
         <ns0:v>0</ns0:v>
       </ns0:c>
-      <ns0:c r="B1" s="14"/>
-      <ns0:c r="C1" s="14"/>
-      <ns0:c r="D1" s="14"/>
-      <ns0:c r="E1" s="14"/>
-      <ns0:c r="F1" s="14"/>
-      <ns0:c r="G1" s="14"/>
-      <ns0:c r="H1" s="14"/>
-      <ns0:c r="I1" s="14"/>
-      <ns0:c r="J1" s="14"/>
-      <ns0:c r="K1" s="14"/>
-      <ns0:c r="L1" s="14"/>
-      <ns0:c r="M1" s="14"/>
-      <ns0:c r="N1" s="14"/>
+      <ns0:c r="B1" s="12"/>
+      <ns0:c r="C1" s="12"/>
+      <ns0:c r="D1" s="12"/>
+      <ns0:c r="E1" s="12"/>
+      <ns0:c r="F1" s="12"/>
+      <ns0:c r="G1" s="12"/>
+      <ns0:c r="H1" s="12"/>
+      <ns0:c r="I1" s="12"/>
+      <ns0:c r="J1" s="12"/>
+      <ns0:c r="K1" s="12"/>
+      <ns0:c r="L1" s="12"/>
+      <ns0:c r="M1" s="12"/>
+      <ns0:c r="N1" s="12"/>
     </ns0:row>
     <ns0:row r="2" spans="1:14" ns3:dyDescent="0.3">
-      <ns0:c r="A2" s="10" t="s">
+      <ns0:c r="A2" s="9" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="B2" s="11" t="inlineStr">
+      <ns0:c r="B2" s="10" t="inlineStr">
         <ns0:is>
           <ns0:t>Abhishek Kumar Vishwakarma</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="E2" s="10" t="s">
+      <ns0:c r="E2" s="9" t="s">
         <ns0:v>3</ns0:v>
       </ns0:c>
-      <ns0:c r="F2" s="11">
+      <ns0:c r="F2" s="10">
         <ns0:v>12617525</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="3" spans="1:14" ns3:dyDescent="0.3">
-      <ns0:c r="A3" s="10" t="s">
+      <ns0:c r="A3" s="9" t="s">
         <ns0:v>4</ns0:v>
       </ns0:c>
-      <ns0:c r="B3" s="12" t="s">
+      <ns0:c r="B3" s="11" t="s">
         <ns0:v>35</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -703,22 +690,22 @@
       <ns0:c r="A4" s="1"/>
     </ns0:row>
     <ns0:row r="5" spans="1:14" ht="61.2" customHeight="1" ns3:dyDescent="0.3">
-      <ns0:c r="A5" s="9" t="s">
+      <ns0:c r="A5" s="8" t="s">
         <ns0:v>5</ns0:v>
       </ns0:c>
-      <ns0:c r="B5" s="9" t="s">
+      <ns0:c r="B5" s="8" t="s">
         <ns0:v>6</ns0:v>
       </ns0:c>
-      <ns0:c r="C5" s="9" t="s">
+      <ns0:c r="C5" s="8" t="s">
         <ns0:v>7</ns0:v>
       </ns0:c>
-      <ns0:c r="D5" s="9" t="s">
+      <ns0:c r="D5" s="8" t="s">
         <ns0:v>8</ns0:v>
       </ns0:c>
-      <ns0:c r="E5" s="9" t="s">
+      <ns0:c r="E5" s="8" t="s">
         <ns0:v>9</ns0:v>
       </ns0:c>
-      <ns0:c r="F5" s="9" t="s">
+      <ns0:c r="F5" s="8" t="s">
         <ns0:v>10</ns0:v>
       </ns0:c>
       <ns0:c r="G5" s="2" t="s">
@@ -2498,49 +2485,93 @@
       <ns0:c r="A44" s="3">
         <ns0:v>46285</ns0:v>
       </ns0:c>
-      <ns0:c r="B44" s="4"/>
-      <ns0:c r="C44" s="13"/>
-      <ns0:c r="D44" s="13"/>
-      <ns0:c r="E44" s="13"/>
-      <ns0:c r="F44" s="13"/>
-      <ns0:c r="G44" s="13"/>
-      <ns0:c r="H44" s="13"/>
-      <ns0:c r="I44" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J44" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K44" s="4"/>
-      <ns0:c r="L44" s="4"/>
-      <ns0:c r="M44" s="4"/>
-      <ns0:c r="N44" s="6"/>
+      <ns0:c r="B44" s="4">
+        <ns0:v>540</ns0:v>
+      </ns0:c>
+      <ns0:c r="C44" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D44" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="E44" s="4">
+        <ns0:v>420</ns0:v>
+      </ns0:c>
+      <ns0:c r="F44" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="G44" s="4">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="H44" s="4">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="I44" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1410</ns0:v>
+      </ns0:c>
+      <ns0:c r="J44" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="K44" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L44" s="4" t="s">
+        <ns0:v>24</ns0:v>
+      </ns0:c>
+      <ns0:c r="M44" s="4" t="s">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="N44" s="4" t="s">
+        <ns0:v>45</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="45" spans="1:14" ht="24" customHeight="1" ns3:dyDescent="0.3">
       <ns0:c r="A45" s="3">
         <ns0:v>46286</ns0:v>
       </ns0:c>
-      <ns0:c r="B45" s="4"/>
-      <ns0:c r="C45" s="13"/>
-      <ns0:c r="D45" s="13"/>
-      <ns0:c r="E45" s="13"/>
-      <ns0:c r="F45" s="13"/>
-      <ns0:c r="G45" s="13"/>
-      <ns0:c r="H45" s="13"/>
-      <ns0:c r="I45" s="5" t="str">
-        <ns0:f t="shared" si="2"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="J45" s="5" t="str">
-        <ns0:f t="shared" si="3"/>
-        <ns0:v/>
-      </ns0:c>
-      <ns0:c r="K45" s="4"/>
-      <ns0:c r="L45" s="4"/>
-      <ns0:c r="M45" s="4"/>
-      <ns0:c r="N45" s="6"/>
+      <ns0:c r="B45" s="4">
+        <ns0:v>540</ns0:v>
+      </ns0:c>
+      <ns0:c r="C45" s="4">
+        <ns0:v>30</ns0:v>
+      </ns0:c>
+      <ns0:c r="D45" s="4">
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="E45" s="4">
+        <ns0:v>120</ns0:v>
+      </ns0:c>
+      <ns0:c r="F45" s="4">
+        <ns0:v>250</ns0:v>
+      </ns0:c>
+      <ns0:c r="G45" s="4">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H45" s="4">
+        <ns0:v>240</ns0:v>
+      </ns0:c>
+      <ns0:c r="I45" s="5">
+        <ns0:f t="shared" si="2"/>
+        <ns0:v>1360</ns0:v>
+      </ns0:c>
+      <ns0:c r="J45" s="5">
+        <ns0:f t="shared" si="3"/>
+        <ns0:v>80</ns0:v>
+      </ns0:c>
+      <ns0:c r="K45" s="4" t="s">
+        <ns0:v>23</ns0:v>
+      </ns0:c>
+      <ns0:c r="L45" s="4" t="s">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="M45" s="4" t="s">
+        <ns0:v>25</ns0:v>
+      </ns0:c>
+      <ns0:c r="N45" s="4" t="s">
+        <ns0:v>46</ns0:v>
+      </ns0:c>
     </ns0:row>
   </ns0:sheetData>
   <ns0:mergeCells count="1">
@@ -2614,110 +2645,110 @@
       <c r="A1" s="1"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="7">
         <v>5</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="7">
         <v>5</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="7">
         <v>4</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="7">
         <v>4</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="7">
         <v>3</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <v>3</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="7">
         <v>2</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="7">
         <v>1</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="7">
         <v>1</v>
       </c>
     </row>

</xml_diff>